<commit_message>
need to add simple ship test and finish updating rng numbers
</commit_message>
<xml_diff>
--- a/shipClassTests/testResults/system_with_subsystems_test.xlsx
+++ b/shipClassTests/testResults/system_with_subsystems_test.xlsx
@@ -407,7 +407,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -415,7 +415,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -423,7 +423,7 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -431,7 +431,7 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -439,7 +439,7 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -447,7 +447,7 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -455,7 +455,7 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -463,7 +463,7 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -471,7 +471,7 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -479,7 +479,7 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -487,7 +487,7 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -495,7 +495,7 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -503,7 +503,7 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -511,7 +511,7 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -519,7 +519,7 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -527,7 +527,7 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -535,7 +535,7 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -559,7 +559,7 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -567,7 +567,7 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -575,7 +575,7 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -583,7 +583,7 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -591,7 +591,7 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -599,7 +599,7 @@
         <v>25</v>
       </c>
       <c r="B27">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -607,7 +607,7 @@
         <v>26</v>
       </c>
       <c r="B28">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -615,7 +615,7 @@
         <v>27</v>
       </c>
       <c r="B29">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -623,7 +623,7 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -631,7 +631,7 @@
         <v>29</v>
       </c>
       <c r="B31">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -639,7 +639,7 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -647,7 +647,7 @@
         <v>31</v>
       </c>
       <c r="B33">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -655,7 +655,7 @@
         <v>32</v>
       </c>
       <c r="B34">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -663,7 +663,7 @@
         <v>33</v>
       </c>
       <c r="B35">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -671,7 +671,7 @@
         <v>34</v>
       </c>
       <c r="B36">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -679,7 +679,7 @@
         <v>35</v>
       </c>
       <c r="B37">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -687,7 +687,7 @@
         <v>36</v>
       </c>
       <c r="B38">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -695,7 +695,7 @@
         <v>37</v>
       </c>
       <c r="B39">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -703,7 +703,7 @@
         <v>38</v>
       </c>
       <c r="B40">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -711,7 +711,7 @@
         <v>39</v>
       </c>
       <c r="B41">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -719,7 +719,7 @@
         <v>40</v>
       </c>
       <c r="B42">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -727,7 +727,7 @@
         <v>41</v>
       </c>
       <c r="B43">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -735,7 +735,7 @@
         <v>42</v>
       </c>
       <c r="B44">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -743,7 +743,7 @@
         <v>43</v>
       </c>
       <c r="B45">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -751,7 +751,7 @@
         <v>44</v>
       </c>
       <c r="B46">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -759,7 +759,7 @@
         <v>45</v>
       </c>
       <c r="B47">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -775,7 +775,7 @@
         <v>47</v>
       </c>
       <c r="B49">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -783,7 +783,7 @@
         <v>48</v>
       </c>
       <c r="B50">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -791,7 +791,7 @@
         <v>49</v>
       </c>
       <c r="B51">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -799,7 +799,7 @@
         <v>50</v>
       </c>
       <c r="B52">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -833,7 +833,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -841,7 +841,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -849,7 +849,7 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -857,7 +857,7 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -865,7 +865,7 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -873,7 +873,7 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -889,7 +889,7 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -905,7 +905,7 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -921,7 +921,7 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -929,7 +929,7 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -937,7 +937,7 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -945,7 +945,7 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -953,7 +953,7 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -961,7 +961,7 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -985,7 +985,7 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -993,7 +993,7 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -1001,7 +1001,7 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -1009,7 +1009,7 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -1017,7 +1017,7 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -1025,7 +1025,7 @@
         <v>25</v>
       </c>
       <c r="B27">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -1033,7 +1033,7 @@
         <v>26</v>
       </c>
       <c r="B28">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -1041,7 +1041,7 @@
         <v>27</v>
       </c>
       <c r="B29">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -1049,7 +1049,7 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -1057,7 +1057,7 @@
         <v>29</v>
       </c>
       <c r="B31">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -1065,7 +1065,7 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -1073,7 +1073,7 @@
         <v>31</v>
       </c>
       <c r="B33">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -1081,7 +1081,7 @@
         <v>32</v>
       </c>
       <c r="B34">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -1089,7 +1089,7 @@
         <v>33</v>
       </c>
       <c r="B35">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -1105,7 +1105,7 @@
         <v>35</v>
       </c>
       <c r="B37">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -1113,7 +1113,7 @@
         <v>36</v>
       </c>
       <c r="B38">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -1129,7 +1129,7 @@
         <v>38</v>
       </c>
       <c r="B40">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -1137,7 +1137,7 @@
         <v>39</v>
       </c>
       <c r="B41">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -1145,7 +1145,7 @@
         <v>40</v>
       </c>
       <c r="B42">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -1153,7 +1153,7 @@
         <v>41</v>
       </c>
       <c r="B43">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -1161,7 +1161,7 @@
         <v>42</v>
       </c>
       <c r="B44">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -1169,7 +1169,7 @@
         <v>43</v>
       </c>
       <c r="B45">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -1177,7 +1177,7 @@
         <v>44</v>
       </c>
       <c r="B46">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -1185,7 +1185,7 @@
         <v>45</v>
       </c>
       <c r="B47">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -1209,7 +1209,7 @@
         <v>48</v>
       </c>
       <c r="B50">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -1217,7 +1217,7 @@
         <v>49</v>
       </c>
       <c r="B51">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -1225,7 +1225,7 @@
         <v>50</v>
       </c>
       <c r="B52">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1259,7 +1259,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1323,7 +1323,7 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -1339,7 +1339,7 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -1379,7 +1379,7 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -1395,7 +1395,7 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -1403,7 +1403,7 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -1443,7 +1443,7 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -1523,7 +1523,7 @@
         <v>34</v>
       </c>
       <c r="B36">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -1531,7 +1531,7 @@
         <v>35</v>
       </c>
       <c r="B37">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -1539,7 +1539,7 @@
         <v>36</v>
       </c>
       <c r="B38">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -1579,7 +1579,7 @@
         <v>41</v>
       </c>
       <c r="B43">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -1619,7 +1619,7 @@
         <v>46</v>
       </c>
       <c r="B48">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -1635,7 +1635,7 @@
         <v>48</v>
       </c>
       <c r="B50">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -1733,7 +1733,7 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1805,7 +1805,7 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -1813,7 +1813,7 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -1821,7 +1821,7 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -1901,7 +1901,7 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -1949,7 +1949,7 @@
         <v>34</v>
       </c>
       <c r="B36">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -1973,7 +1973,7 @@
         <v>37</v>
       </c>
       <c r="B39">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -2111,7 +2111,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -2119,7 +2119,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -2127,7 +2127,7 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -2135,7 +2135,7 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -2143,7 +2143,7 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -2151,7 +2151,7 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -2159,7 +2159,7 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -2167,7 +2167,7 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -2175,7 +2175,7 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -2183,7 +2183,7 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -2191,7 +2191,7 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -2199,7 +2199,7 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -2207,7 +2207,7 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -2215,7 +2215,7 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -2223,7 +2223,7 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -2231,7 +2231,7 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -2239,7 +2239,7 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -2247,7 +2247,7 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -2255,7 +2255,7 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -2263,7 +2263,7 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -2271,7 +2271,7 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -2279,7 +2279,7 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -2287,7 +2287,7 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -2295,7 +2295,7 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -2303,7 +2303,7 @@
         <v>25</v>
       </c>
       <c r="B27">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -2311,7 +2311,7 @@
         <v>26</v>
       </c>
       <c r="B28">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -2319,7 +2319,7 @@
         <v>27</v>
       </c>
       <c r="B29">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -2327,7 +2327,7 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -2335,7 +2335,7 @@
         <v>29</v>
       </c>
       <c r="B31">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -2343,7 +2343,7 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -2351,7 +2351,7 @@
         <v>31</v>
       </c>
       <c r="B33">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -2359,7 +2359,7 @@
         <v>32</v>
       </c>
       <c r="B34">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -2367,7 +2367,7 @@
         <v>33</v>
       </c>
       <c r="B35">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -2375,7 +2375,7 @@
         <v>34</v>
       </c>
       <c r="B36">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -2383,7 +2383,7 @@
         <v>35</v>
       </c>
       <c r="B37">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -2391,7 +2391,7 @@
         <v>36</v>
       </c>
       <c r="B38">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -2399,7 +2399,7 @@
         <v>37</v>
       </c>
       <c r="B39">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -2407,7 +2407,7 @@
         <v>38</v>
       </c>
       <c r="B40">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -2415,7 +2415,7 @@
         <v>39</v>
       </c>
       <c r="B41">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -2423,7 +2423,7 @@
         <v>40</v>
       </c>
       <c r="B42">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -2431,7 +2431,7 @@
         <v>41</v>
       </c>
       <c r="B43">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -2439,7 +2439,7 @@
         <v>42</v>
       </c>
       <c r="B44">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -2447,7 +2447,7 @@
         <v>43</v>
       </c>
       <c r="B45">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -2455,7 +2455,7 @@
         <v>44</v>
       </c>
       <c r="B46">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -2463,7 +2463,7 @@
         <v>45</v>
       </c>
       <c r="B47">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -2471,7 +2471,7 @@
         <v>46</v>
       </c>
       <c r="B48">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -2487,7 +2487,7 @@
         <v>48</v>
       </c>
       <c r="B50">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -2495,7 +2495,7 @@
         <v>49</v>
       </c>
       <c r="B51">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -2503,7 +2503,7 @@
         <v>50</v>
       </c>
       <c r="B52">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2537,7 +2537,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -2545,7 +2545,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -2553,7 +2553,7 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -2561,7 +2561,7 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -2569,7 +2569,7 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -2585,7 +2585,7 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -2593,7 +2593,7 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -2601,7 +2601,7 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -2609,7 +2609,7 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -2617,7 +2617,7 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -2625,7 +2625,7 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -2633,7 +2633,7 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -2641,7 +2641,7 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -2649,7 +2649,7 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -2657,7 +2657,7 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -2689,7 +2689,7 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -2705,7 +2705,7 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -2713,7 +2713,7 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -2721,7 +2721,7 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -2729,7 +2729,7 @@
         <v>25</v>
       </c>
       <c r="B27">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -2753,7 +2753,7 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -2801,7 +2801,7 @@
         <v>34</v>
       </c>
       <c r="B36">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -2809,7 +2809,7 @@
         <v>35</v>
       </c>
       <c r="B37">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -2817,7 +2817,7 @@
         <v>36</v>
       </c>
       <c r="B38">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -2825,7 +2825,7 @@
         <v>37</v>
       </c>
       <c r="B39">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -2833,7 +2833,7 @@
         <v>38</v>
       </c>
       <c r="B40">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -2841,7 +2841,7 @@
         <v>39</v>
       </c>
       <c r="B41">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -2849,7 +2849,7 @@
         <v>40</v>
       </c>
       <c r="B42">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -2857,7 +2857,7 @@
         <v>41</v>
       </c>
       <c r="B43">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -2865,7 +2865,7 @@
         <v>42</v>
       </c>
       <c r="B44">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -2873,7 +2873,7 @@
         <v>43</v>
       </c>
       <c r="B45">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -2881,7 +2881,7 @@
         <v>44</v>
       </c>
       <c r="B46">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -2889,7 +2889,7 @@
         <v>45</v>
       </c>
       <c r="B47">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -2905,7 +2905,7 @@
         <v>47</v>
       </c>
       <c r="B49">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -2913,7 +2913,7 @@
         <v>48</v>
       </c>
       <c r="B50">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -2929,7 +2929,7 @@
         <v>50</v>
       </c>
       <c r="B52">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3011,7 +3011,7 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -3019,7 +3019,7 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -3027,7 +3027,7 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -3035,7 +3035,7 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -3043,7 +3043,7 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -3051,7 +3051,7 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -3083,7 +3083,7 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -3091,7 +3091,7 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -3107,7 +3107,7 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -3115,7 +3115,7 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -3123,7 +3123,7 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -3131,7 +3131,7 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -3139,7 +3139,7 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -3147,7 +3147,7 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -3155,7 +3155,7 @@
         <v>25</v>
       </c>
       <c r="B27">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -3171,7 +3171,7 @@
         <v>27</v>
       </c>
       <c r="B29">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -3179,7 +3179,7 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -3187,7 +3187,7 @@
         <v>29</v>
       </c>
       <c r="B31">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -3195,7 +3195,7 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -3203,7 +3203,7 @@
         <v>31</v>
       </c>
       <c r="B33">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -3211,7 +3211,7 @@
         <v>32</v>
       </c>
       <c r="B34">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -3219,7 +3219,7 @@
         <v>33</v>
       </c>
       <c r="B35">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -3227,7 +3227,7 @@
         <v>34</v>
       </c>
       <c r="B36">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -3235,7 +3235,7 @@
         <v>35</v>
       </c>
       <c r="B37">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -3243,7 +3243,7 @@
         <v>36</v>
       </c>
       <c r="B38">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -3251,7 +3251,7 @@
         <v>37</v>
       </c>
       <c r="B39">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -3259,7 +3259,7 @@
         <v>38</v>
       </c>
       <c r="B40">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -3267,7 +3267,7 @@
         <v>39</v>
       </c>
       <c r="B41">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -3275,7 +3275,7 @@
         <v>40</v>
       </c>
       <c r="B42">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -3283,7 +3283,7 @@
         <v>41</v>
       </c>
       <c r="B43">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -3291,7 +3291,7 @@
         <v>42</v>
       </c>
       <c r="B44">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -3299,7 +3299,7 @@
         <v>43</v>
       </c>
       <c r="B45">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -3307,7 +3307,7 @@
         <v>44</v>
       </c>
       <c r="B46">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -3315,7 +3315,7 @@
         <v>45</v>
       </c>
       <c r="B47">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -3323,7 +3323,7 @@
         <v>46</v>
       </c>
       <c r="B48">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -3331,7 +3331,7 @@
         <v>47</v>
       </c>
       <c r="B49">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -3339,7 +3339,7 @@
         <v>48</v>
       </c>
       <c r="B50">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -3347,7 +3347,7 @@
         <v>49</v>
       </c>
       <c r="B51">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -3355,7 +3355,7 @@
         <v>50</v>
       </c>
       <c r="B52">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -3389,7 +3389,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -3397,7 +3397,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -3413,7 +3413,7 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -3421,7 +3421,7 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -3429,7 +3429,7 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -3437,7 +3437,7 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -3445,7 +3445,7 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -3453,7 +3453,7 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -3461,7 +3461,7 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -3469,7 +3469,7 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -3477,7 +3477,7 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -3485,7 +3485,7 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -3493,7 +3493,7 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -3501,7 +3501,7 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -3509,7 +3509,7 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -3517,7 +3517,7 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -3525,7 +3525,7 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -3533,7 +3533,7 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -3541,7 +3541,7 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -3549,7 +3549,7 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -3557,7 +3557,7 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -3565,7 +3565,7 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -3573,7 +3573,7 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -3581,7 +3581,7 @@
         <v>25</v>
       </c>
       <c r="B27">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -3589,7 +3589,7 @@
         <v>26</v>
       </c>
       <c r="B28">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -3597,7 +3597,7 @@
         <v>27</v>
       </c>
       <c r="B29">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -3605,7 +3605,7 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -3613,7 +3613,7 @@
         <v>29</v>
       </c>
       <c r="B31">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -3621,7 +3621,7 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -3629,7 +3629,7 @@
         <v>31</v>
       </c>
       <c r="B33">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -3637,7 +3637,7 @@
         <v>32</v>
       </c>
       <c r="B34">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -3645,7 +3645,7 @@
         <v>33</v>
       </c>
       <c r="B35">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -3653,7 +3653,7 @@
         <v>34</v>
       </c>
       <c r="B36">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -3661,7 +3661,7 @@
         <v>35</v>
       </c>
       <c r="B37">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -3669,7 +3669,7 @@
         <v>36</v>
       </c>
       <c r="B38">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -3677,7 +3677,7 @@
         <v>37</v>
       </c>
       <c r="B39">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -3685,7 +3685,7 @@
         <v>38</v>
       </c>
       <c r="B40">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -3693,7 +3693,7 @@
         <v>39</v>
       </c>
       <c r="B41">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -3701,7 +3701,7 @@
         <v>40</v>
       </c>
       <c r="B42">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -3709,7 +3709,7 @@
         <v>41</v>
       </c>
       <c r="B43">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -3717,7 +3717,7 @@
         <v>42</v>
       </c>
       <c r="B44">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -3725,7 +3725,7 @@
         <v>43</v>
       </c>
       <c r="B45">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -3733,7 +3733,7 @@
         <v>44</v>
       </c>
       <c r="B46">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -3741,7 +3741,7 @@
         <v>45</v>
       </c>
       <c r="B47">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -3749,7 +3749,7 @@
         <v>46</v>
       </c>
       <c r="B48">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -3757,7 +3757,7 @@
         <v>47</v>
       </c>
       <c r="B49">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -3765,7 +3765,7 @@
         <v>48</v>
       </c>
       <c r="B50">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -3781,7 +3781,7 @@
         <v>50</v>
       </c>
       <c r="B52">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -3823,7 +3823,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -3831,7 +3831,7 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -3839,7 +3839,7 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -3847,7 +3847,7 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -3855,7 +3855,7 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -3911,7 +3911,7 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -3919,7 +3919,7 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -3927,7 +3927,7 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -3935,7 +3935,7 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -3967,7 +3967,7 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -3983,7 +3983,7 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -3991,7 +3991,7 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -3999,7 +3999,7 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -4007,7 +4007,7 @@
         <v>25</v>
       </c>
       <c r="B27">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -4015,7 +4015,7 @@
         <v>26</v>
       </c>
       <c r="B28">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -4031,7 +4031,7 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -4079,7 +4079,7 @@
         <v>34</v>
       </c>
       <c r="B36">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -4087,7 +4087,7 @@
         <v>35</v>
       </c>
       <c r="B37">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -4095,7 +4095,7 @@
         <v>36</v>
       </c>
       <c r="B38">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -4103,7 +4103,7 @@
         <v>37</v>
       </c>
       <c r="B39">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -4111,7 +4111,7 @@
         <v>38</v>
       </c>
       <c r="B40">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -4119,7 +4119,7 @@
         <v>39</v>
       </c>
       <c r="B41">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -4127,7 +4127,7 @@
         <v>40</v>
       </c>
       <c r="B42">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -4135,7 +4135,7 @@
         <v>41</v>
       </c>
       <c r="B43">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -4143,7 +4143,7 @@
         <v>42</v>
       </c>
       <c r="B44">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -4151,7 +4151,7 @@
         <v>43</v>
       </c>
       <c r="B45">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -4159,7 +4159,7 @@
         <v>44</v>
       </c>
       <c r="B46">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -4167,7 +4167,7 @@
         <v>45</v>
       </c>
       <c r="B47">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -4183,7 +4183,7 @@
         <v>47</v>
       </c>
       <c r="B49">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -4191,7 +4191,7 @@
         <v>48</v>
       </c>
       <c r="B50">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -4199,7 +4199,7 @@
         <v>49</v>
       </c>
       <c r="B51">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -4207,7 +4207,7 @@
         <v>50</v>
       </c>
       <c r="B52">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>